<commit_message>
modify stm32 source ic
</commit_message>
<xml_diff>
--- a/fnrisV0_1/fNIRS_V0_1-STM32/document/通信指令.xlsx
+++ b/fnrisV0_1/fNIRS_V0_1-STM32/document/通信指令.xlsx
@@ -441,7 +441,7 @@
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FFC00000"/>
+      <color theme="5" tint="-0.25"/>
       <name val="宋体"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -455,7 +455,7 @@
     </font>
     <font>
       <sz val="11"/>
-      <color theme="5" tint="-0.25"/>
+      <color rgb="FFC00000"/>
       <name val="宋体"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -620,30 +620,66 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFC00000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B0F0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor theme="4" tint="0.8"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor theme="4" tint="0.6"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF00B0F0"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC000"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="6" tint="-0.25"/>
         <bgColor indexed="64"/>
       </patternFill>
@@ -651,42 +687,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="4" tint="0.4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC00000"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF92D050"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF00B050"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -910,6 +910,21 @@
       <diagonal/>
     </border>
     <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thick">
+        <color auto="1"/>
+      </right>
+      <top style="thick">
+        <color auto="1"/>
+      </top>
+      <bottom style="thick">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left style="thick">
         <color auto="1"/>
       </left>
@@ -923,6 +938,21 @@
       <diagonal/>
     </border>
     <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left style="thick">
         <color auto="1"/>
       </left>
@@ -979,6 +1009,49 @@
       <diagonal/>
     </border>
     <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thick">
+        <color auto="1"/>
+      </right>
+      <top style="thick">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="dashed">
+        <color auto="1"/>
+      </left>
+      <right style="dashed">
+        <color auto="1"/>
+      </right>
+      <top style="dashed">
+        <color auto="1"/>
+      </top>
+      <bottom style="dashed">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="dashed">
+        <color auto="1"/>
+      </left>
+      <right style="dashed">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom style="dashed">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left style="thick">
         <color auto="1"/>
       </left>
@@ -1022,6 +1095,65 @@
       <diagonal/>
     </border>
     <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thick">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="dashed">
+        <color auto="1"/>
+      </left>
+      <right style="dashed">
+        <color auto="1"/>
+      </right>
+      <top style="dashed">
+        <color auto="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="double">
+        <color auto="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="hair">
+        <color auto="1"/>
+      </left>
+      <right style="hair">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom style="hair">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left style="thick">
         <color auto="1"/>
       </left>
@@ -1060,6 +1192,36 @@
         <color auto="1"/>
       </top>
       <bottom style="thick">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thick">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thick">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="hair">
+        <color auto="1"/>
+      </left>
+      <right style="hair">
+        <color auto="1"/>
+      </right>
+      <top style="hair">
+        <color auto="1"/>
+      </top>
+      <bottom style="hair">
         <color auto="1"/>
       </bottom>
       <diagonal/>
@@ -1117,6 +1279,26 @@
       <diagonal/>
     </border>
     <border>
+      <left/>
+      <right style="thick">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thick">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom style="thick">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left style="thick">
         <color auto="1"/>
       </left>
@@ -1135,6 +1317,30 @@
       <top style="thick">
         <color auto="1"/>
       </top>
+      <bottom style="thick">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thick">
+        <color auto="1"/>
+      </right>
+      <top style="thick">
+        <color auto="1"/>
+      </top>
+      <bottom style="thick">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thick">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top/>
       <bottom style="thick">
         <color auto="1"/>
       </bottom>
@@ -1170,21 +1376,6 @@
       <diagonal/>
     </border>
     <border>
-      <left style="dashed">
-        <color auto="1"/>
-      </left>
-      <right style="dashed">
-        <color auto="1"/>
-      </right>
-      <top style="dashed">
-        <color auto="1"/>
-      </top>
-      <bottom style="dashed">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left style="hair">
         <color auto="1"/>
       </left>
@@ -1204,197 +1395,6 @@
         <color auto="1"/>
       </top>
       <bottom style="hair">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="hair">
-        <color auto="1"/>
-      </left>
-      <right style="hair">
-        <color auto="1"/>
-      </right>
-      <top style="hair">
-        <color auto="1"/>
-      </top>
-      <bottom style="hair">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thick">
-        <color auto="1"/>
-      </right>
-      <top style="thick">
-        <color auto="1"/>
-      </top>
-      <bottom style="thick">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color auto="1"/>
-      </left>
-      <right style="medium">
-        <color auto="1"/>
-      </right>
-      <top style="medium">
-        <color auto="1"/>
-      </top>
-      <bottom style="medium">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thick">
-        <color auto="1"/>
-      </right>
-      <top style="thick">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="dashed">
-        <color auto="1"/>
-      </left>
-      <right style="dashed">
-        <color auto="1"/>
-      </right>
-      <top/>
-      <bottom style="dashed">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thick">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="hair">
-        <color auto="1"/>
-      </left>
-      <right style="hair">
-        <color auto="1"/>
-      </right>
-      <top/>
-      <bottom style="hair">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thick">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thick">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thick">
-        <color auto="1"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thick">
-        <color auto="1"/>
-      </right>
-      <top/>
-      <bottom style="thick">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thick">
-        <color auto="1"/>
-      </right>
-      <top style="thick">
-        <color auto="1"/>
-      </top>
-      <bottom style="thick">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thick">
-        <color auto="1"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom style="thick">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="dashed">
-        <color auto="1"/>
-      </left>
-      <right style="dashed">
-        <color auto="1"/>
-      </right>
-      <top style="dashed">
-        <color auto="1"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="double">
-        <color auto="1"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="double">
         <color auto="1"/>
       </bottom>
       <diagonal/>
@@ -1623,7 +1623,7 @@
     <xf numFmtId="0" fontId="25" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="26" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1673,286 +1673,286 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="23" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="23" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="24" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="29" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="22" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="30" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="31" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="58" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="35" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="36" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="37" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="38" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="37" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="14" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="39" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="40" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="28" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="28" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="11" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="29" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="30" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="31" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="23" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="23" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="23" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="33" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="34" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="35" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="37" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="35" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="28" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="28" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="28" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="30" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="30" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="23" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="23" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="38" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="38" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="38" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="58" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="41" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" quotePrefix="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="23" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" quotePrefix="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" quotePrefix="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" quotePrefix="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -2403,7 +2403,7 @@
     <col min="24" max="16384" width="9" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" ht="33" customHeight="1" spans="1:11">
+    <row r="1" ht="33" customHeight="1" spans="1:23">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -2416,1033 +2416,1033 @@
       <c r="H1" s="3"/>
       <c r="I1" s="3"/>
       <c r="J1" s="3"/>
-      <c r="K1" s="51"/>
-    </row>
-    <row r="2" s="1" customFormat="1" ht="48" customHeight="1" spans="1:16">
+      <c r="K1" s="4"/>
+    </row>
+    <row r="2" s="1" customFormat="1" ht="48" customHeight="1" spans="1:23">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="K2" s="52"/>
-      <c r="L2" s="53"/>
-      <c r="M2" s="54"/>
-      <c r="N2" s="54"/>
-      <c r="O2" s="54"/>
-      <c r="P2" s="54"/>
-    </row>
-    <row r="3" s="1" customFormat="1" ht="15" spans="1:16">
-      <c r="A3" s="4" t="s">
+      <c r="K2" s="5"/>
+      <c r="L2" s="6"/>
+      <c r="M2" s="7"/>
+      <c r="N2" s="7"/>
+      <c r="O2" s="7"/>
+      <c r="P2" s="7"/>
+    </row>
+    <row r="3" s="1" customFormat="1" ht="15" spans="1:23">
+      <c r="A3" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="5"/>
-      <c r="C3" s="5"/>
-      <c r="D3" s="5"/>
-      <c r="E3" s="5"/>
-      <c r="F3" s="5"/>
-      <c r="G3" s="5"/>
-      <c r="H3" s="5"/>
-      <c r="I3" s="5"/>
-      <c r="J3" s="55"/>
-      <c r="K3" s="52"/>
-      <c r="L3" s="53"/>
-      <c r="M3" s="54" t="s">
+      <c r="B3" s="9"/>
+      <c r="C3" s="9"/>
+      <c r="D3" s="9"/>
+      <c r="E3" s="9"/>
+      <c r="F3" s="9"/>
+      <c r="G3" s="9"/>
+      <c r="H3" s="9"/>
+      <c r="I3" s="9"/>
+      <c r="J3" s="10"/>
+      <c r="K3" s="5"/>
+      <c r="L3" s="6"/>
+      <c r="M3" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="N3" s="54"/>
-      <c r="O3" s="54"/>
-      <c r="P3" s="54"/>
+      <c r="N3" s="7"/>
+      <c r="O3" s="7"/>
+      <c r="P3" s="7"/>
     </row>
     <row r="4" ht="15" spans="1:23">
-      <c r="A4" s="6"/>
-      <c r="B4" s="6" t="s">
+      <c r="A4" s="11"/>
+      <c r="B4" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="C4" s="6" t="s">
+      <c r="C4" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="D4" s="6" t="s">
+      <c r="D4" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="E4" s="6" t="s">
+      <c r="E4" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="F4" s="6" t="s">
+      <c r="F4" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="G4" s="6" t="s">
+      <c r="G4" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="H4" s="6"/>
-      <c r="I4" s="6"/>
-      <c r="J4" s="6" t="s">
+      <c r="H4" s="11"/>
+      <c r="I4" s="11"/>
+      <c r="J4" s="11" t="s">
         <v>10</v>
       </c>
-      <c r="L4" s="56"/>
-      <c r="M4" s="57" t="s">
+      <c r="L4" s="12"/>
+      <c r="M4" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="N4" s="57"/>
-      <c r="O4" s="57"/>
-      <c r="P4" s="57"/>
-      <c r="R4" s="82" t="s">
+      <c r="N4" s="13"/>
+      <c r="O4" s="13"/>
+      <c r="P4" s="13"/>
+      <c r="R4" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="S4" s="82"/>
-      <c r="T4" s="82"/>
-      <c r="U4" s="82"/>
-      <c r="V4" s="82"/>
-      <c r="W4" s="82"/>
+      <c r="S4" s="14"/>
+      <c r="T4" s="14"/>
+      <c r="U4" s="14"/>
+      <c r="V4" s="14"/>
+      <c r="W4" s="14"/>
     </row>
     <row r="5" ht="15" spans="1:23">
-      <c r="A5" s="7"/>
-      <c r="B5" s="8" t="s">
+      <c r="A5" s="15"/>
+      <c r="B5" s="16" t="s">
         <v>13</v>
       </c>
-      <c r="C5" s="8" t="s">
+      <c r="C5" s="16" t="s">
         <v>14</v>
       </c>
-      <c r="D5" s="8" t="s">
+      <c r="D5" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="E5" s="8" t="s">
+      <c r="E5" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="F5" s="8" t="s">
+      <c r="F5" s="16" t="s">
         <v>13</v>
       </c>
-      <c r="G5" s="8" t="s">
+      <c r="G5" s="16" t="s">
         <v>16</v>
       </c>
-      <c r="H5" s="8"/>
-      <c r="I5" s="8"/>
-      <c r="J5" s="8" t="s">
+      <c r="H5" s="16"/>
+      <c r="I5" s="16"/>
+      <c r="J5" s="16" t="s">
         <v>13</v>
       </c>
-      <c r="L5" s="56"/>
-      <c r="M5" s="58" t="s">
+      <c r="L5" s="12"/>
+      <c r="M5" s="17" t="s">
         <v>17</v>
       </c>
-      <c r="N5" s="58"/>
-      <c r="O5" s="59" t="s">
+      <c r="N5" s="17"/>
+      <c r="O5" s="18" t="s">
         <v>18</v>
       </c>
-      <c r="P5" s="59"/>
-      <c r="R5" s="58" t="s">
+      <c r="P5" s="18"/>
+      <c r="R5" s="17" t="s">
         <v>17</v>
       </c>
-      <c r="S5" s="83" t="s">
+      <c r="S5" s="19" t="s">
         <v>19</v>
       </c>
-      <c r="T5" s="83"/>
-      <c r="U5" s="84" t="s">
+      <c r="T5" s="19"/>
+      <c r="U5" s="20" t="s">
         <v>20</v>
       </c>
-      <c r="V5" s="84"/>
-      <c r="W5" s="84"/>
+      <c r="V5" s="20"/>
+      <c r="W5" s="20"/>
     </row>
     <row r="6" ht="15" spans="1:23">
-      <c r="A6" s="9" t="s">
+      <c r="A6" s="21" t="s">
         <v>21</v>
       </c>
-      <c r="B6" s="10" t="s">
+      <c r="B6" s="22" t="s">
         <v>22</v>
       </c>
       <c r="C6" s="96" t="s">
         <v>23</v>
       </c>
-      <c r="D6" s="12" t="s">
+      <c r="D6" s="24" t="s">
         <v>24</v>
       </c>
-      <c r="E6" s="13" t="s">
+      <c r="E6" s="25" t="s">
         <v>25</v>
       </c>
-      <c r="F6" s="13">
+      <c r="F6" s="25">
         <v>4</v>
       </c>
-      <c r="G6" s="13" t="s">
+      <c r="G6" s="25" t="s">
         <v>26</v>
       </c>
-      <c r="H6" s="13"/>
-      <c r="I6" s="13"/>
-      <c r="J6" s="60" t="s">
+      <c r="H6" s="25"/>
+      <c r="I6" s="25"/>
+      <c r="J6" s="26" t="s">
         <v>27</v>
       </c>
-      <c r="L6" s="61"/>
-      <c r="M6" s="62" t="s">
+      <c r="L6" s="27"/>
+      <c r="M6" s="28" t="s">
         <v>28</v>
       </c>
-      <c r="N6" s="62"/>
-      <c r="O6" s="62"/>
-      <c r="P6" s="62"/>
-      <c r="R6" s="62" t="s">
+      <c r="N6" s="28"/>
+      <c r="O6" s="28"/>
+      <c r="P6" s="28"/>
+      <c r="R6" s="28" t="s">
         <v>29</v>
       </c>
-      <c r="S6" s="85" t="s">
+      <c r="S6" s="29" t="s">
         <v>30</v>
       </c>
-      <c r="T6" s="85"/>
-      <c r="U6" s="86" t="s">
+      <c r="T6" s="29"/>
+      <c r="U6" s="30" t="s">
         <v>31</v>
       </c>
-      <c r="V6" s="86"/>
-      <c r="W6" s="86"/>
+      <c r="V6" s="30"/>
+      <c r="W6" s="30"/>
     </row>
     <row r="7" ht="14.25" spans="1:23">
-      <c r="A7" s="14" t="s">
+      <c r="A7" s="31" t="s">
         <v>32</v>
       </c>
-      <c r="B7" s="15"/>
-      <c r="C7" s="16" t="s">
+      <c r="B7" s="32"/>
+      <c r="C7" s="33" t="s">
         <v>33</v>
       </c>
-      <c r="D7" s="17"/>
-      <c r="E7" s="18" t="s">
+      <c r="D7" s="34"/>
+      <c r="E7" s="35" t="s">
         <v>34</v>
       </c>
-      <c r="F7" s="18">
+      <c r="F7" s="35">
         <v>0</v>
       </c>
-      <c r="G7" s="18" t="s">
+      <c r="G7" s="35" t="s">
         <v>35</v>
       </c>
-      <c r="H7" s="18"/>
-      <c r="I7" s="18"/>
-      <c r="J7" s="63"/>
-      <c r="L7" s="64" t="s">
+      <c r="H7" s="35"/>
+      <c r="I7" s="35"/>
+      <c r="J7" s="36"/>
+      <c r="L7" s="37" t="s">
         <v>36</v>
       </c>
-      <c r="M7" s="65" t="s">
+      <c r="M7" s="38" t="s">
         <v>29</v>
       </c>
-      <c r="N7" s="65" t="s">
+      <c r="N7" s="38" t="s">
         <v>37</v>
       </c>
-      <c r="O7" s="65" t="s">
+      <c r="O7" s="38" t="s">
         <v>38</v>
       </c>
-      <c r="P7" s="65" t="s">
+      <c r="P7" s="38" t="s">
         <v>39</v>
       </c>
-      <c r="R7" s="65" t="s">
+      <c r="R7" s="38" t="s">
         <v>37</v>
       </c>
-      <c r="S7" s="87" t="s">
+      <c r="S7" s="39" t="s">
         <v>30</v>
       </c>
-      <c r="T7" s="87"/>
-      <c r="U7" s="88" t="s">
+      <c r="T7" s="39"/>
+      <c r="U7" s="40" t="s">
         <v>31</v>
       </c>
-      <c r="V7" s="88"/>
-      <c r="W7" s="88"/>
+      <c r="V7" s="40"/>
+      <c r="W7" s="40"/>
     </row>
     <row r="8" ht="14.25" spans="1:23">
-      <c r="A8" s="14" t="s">
+      <c r="A8" s="31" t="s">
         <v>40</v>
       </c>
-      <c r="B8" s="15"/>
-      <c r="C8" s="16"/>
-      <c r="D8" s="17"/>
-      <c r="E8" s="18" t="s">
+      <c r="B8" s="32"/>
+      <c r="C8" s="33"/>
+      <c r="D8" s="34"/>
+      <c r="E8" s="35" t="s">
         <v>41</v>
       </c>
-      <c r="F8" s="18">
+      <c r="F8" s="35">
         <v>0</v>
       </c>
-      <c r="G8" s="18" t="s">
+      <c r="G8" s="35" t="s">
         <v>35</v>
       </c>
-      <c r="H8" s="18"/>
-      <c r="I8" s="18"/>
-      <c r="J8" s="63"/>
+      <c r="H8" s="35"/>
+      <c r="I8" s="35"/>
+      <c r="J8" s="36"/>
       <c r="L8" s="97" t="s">
         <v>42</v>
       </c>
-      <c r="M8" s="67">
+      <c r="M8" s="42">
         <v>500</v>
       </c>
-      <c r="N8" s="67">
+      <c r="N8" s="42">
         <v>500</v>
       </c>
-      <c r="O8" s="67">
+      <c r="O8" s="42">
         <v>10</v>
       </c>
-      <c r="P8" s="67">
+      <c r="P8" s="42">
         <v>10</v>
       </c>
-      <c r="R8" s="65" t="s">
+      <c r="R8" s="38" t="s">
         <v>38</v>
       </c>
-      <c r="S8" s="87" t="s">
+      <c r="S8" s="39" t="s">
         <v>43</v>
       </c>
-      <c r="T8" s="87" t="s">
+      <c r="T8" s="39" t="s">
         <v>44</v>
       </c>
-      <c r="U8" s="88" t="s">
+      <c r="U8" s="40" t="s">
         <v>45</v>
       </c>
-      <c r="V8" s="88" t="s">
+      <c r="V8" s="40" t="s">
         <v>46</v>
       </c>
-      <c r="W8" s="88" t="s">
+      <c r="W8" s="40" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="9" ht="14.25" spans="1:23">
-      <c r="A9" s="14" t="s">
+      <c r="A9" s="31" t="s">
         <v>48</v>
       </c>
-      <c r="B9" s="15"/>
-      <c r="C9" s="16"/>
-      <c r="D9" s="17"/>
-      <c r="E9" s="18" t="s">
+      <c r="B9" s="32"/>
+      <c r="C9" s="33"/>
+      <c r="D9" s="34"/>
+      <c r="E9" s="35" t="s">
         <v>49</v>
       </c>
-      <c r="F9" s="18">
+      <c r="F9" s="35">
         <v>0</v>
       </c>
-      <c r="G9" s="18" t="s">
+      <c r="G9" s="35" t="s">
         <v>35</v>
       </c>
-      <c r="H9" s="18"/>
-      <c r="I9" s="18"/>
-      <c r="J9" s="63"/>
+      <c r="H9" s="35"/>
+      <c r="I9" s="35"/>
+      <c r="J9" s="36"/>
       <c r="L9" s="97" t="s">
         <v>50</v>
       </c>
-      <c r="M9" s="67">
+      <c r="M9" s="42">
         <v>1000</v>
       </c>
-      <c r="N9" s="67">
+      <c r="N9" s="42">
         <v>1000</v>
       </c>
-      <c r="O9" s="67">
+      <c r="O9" s="42">
         <v>20</v>
       </c>
-      <c r="P9" s="67">
+      <c r="P9" s="42">
         <v>20</v>
       </c>
-      <c r="R9" s="89" t="s">
+      <c r="R9" s="43" t="s">
         <v>39</v>
       </c>
-      <c r="S9" s="90" t="s">
+      <c r="S9" s="44" t="s">
         <v>43</v>
       </c>
-      <c r="T9" s="90" t="s">
+      <c r="T9" s="44" t="s">
         <v>44</v>
       </c>
-      <c r="U9" s="91" t="s">
+      <c r="U9" s="45" t="s">
         <v>45</v>
       </c>
-      <c r="V9" s="91" t="s">
+      <c r="V9" s="45" t="s">
         <v>46</v>
       </c>
-      <c r="W9" s="91" t="s">
+      <c r="W9" s="45" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="10" ht="15" spans="1:23">
-      <c r="A10" s="14" t="s">
+      <c r="A10" s="31" t="s">
         <v>51</v>
       </c>
-      <c r="B10" s="15"/>
-      <c r="C10" s="16"/>
-      <c r="D10" s="17"/>
-      <c r="E10" s="18" t="s">
+      <c r="B10" s="32"/>
+      <c r="C10" s="33"/>
+      <c r="D10" s="34"/>
+      <c r="E10" s="35" t="s">
         <v>52</v>
       </c>
-      <c r="F10" s="18">
+      <c r="F10" s="35">
         <v>0</v>
       </c>
-      <c r="G10" s="18" t="s">
+      <c r="G10" s="35" t="s">
         <v>35</v>
       </c>
-      <c r="H10" s="18"/>
-      <c r="I10" s="18"/>
-      <c r="J10" s="63"/>
+      <c r="H10" s="35"/>
+      <c r="I10" s="35"/>
+      <c r="J10" s="36"/>
       <c r="L10" s="97" t="s">
         <v>53</v>
       </c>
-      <c r="M10" s="67">
+      <c r="M10" s="42">
         <v>2000</v>
       </c>
-      <c r="N10" s="67">
+      <c r="N10" s="42">
         <v>2000</v>
       </c>
-      <c r="O10" s="67" t="s">
+      <c r="O10" s="42" t="s">
         <v>35</v>
       </c>
-      <c r="P10" s="67">
+      <c r="P10" s="42">
         <v>40</v>
       </c>
-      <c r="R10" s="92" t="s">
+      <c r="R10" s="46" t="s">
         <v>54</v>
       </c>
-      <c r="S10" s="92"/>
-      <c r="T10" s="92"/>
-      <c r="U10" s="92"/>
-      <c r="V10" s="92"/>
-      <c r="W10" s="92"/>
+      <c r="S10" s="46"/>
+      <c r="T10" s="46"/>
+      <c r="U10" s="46"/>
+      <c r="V10" s="46"/>
+      <c r="W10" s="46"/>
     </row>
     <row r="11" ht="14.25" spans="1:23">
-      <c r="A11" s="14" t="s">
+      <c r="A11" s="31" t="s">
         <v>55</v>
       </c>
-      <c r="B11" s="15"/>
-      <c r="C11" s="16"/>
-      <c r="D11" s="17"/>
-      <c r="E11" s="18" t="s">
+      <c r="B11" s="32"/>
+      <c r="C11" s="33"/>
+      <c r="D11" s="34"/>
+      <c r="E11" s="35" t="s">
         <v>56</v>
       </c>
-      <c r="F11" s="18" t="s">
+      <c r="F11" s="35" t="s">
         <v>57</v>
       </c>
-      <c r="G11" s="19" t="s">
+      <c r="G11" s="47" t="s">
         <v>58</v>
       </c>
-      <c r="H11" s="18" t="s">
+      <c r="H11" s="35" t="s">
         <v>46</v>
       </c>
-      <c r="I11" s="19" t="s">
+      <c r="I11" s="47" t="s">
         <v>11</v>
       </c>
-      <c r="J11" s="63"/>
+      <c r="J11" s="36"/>
       <c r="L11" s="97" t="s">
         <v>59</v>
       </c>
-      <c r="M11" s="67">
+      <c r="M11" s="42">
         <v>4000</v>
       </c>
-      <c r="N11" s="67">
+      <c r="N11" s="42">
         <v>4000</v>
       </c>
-      <c r="O11" s="67" t="s">
+      <c r="O11" s="42" t="s">
         <v>35</v>
       </c>
-      <c r="P11" s="67">
+      <c r="P11" s="42">
         <v>80</v>
       </c>
-      <c r="R11" s="93" t="s">
+      <c r="R11" s="48" t="s">
         <v>60</v>
       </c>
-      <c r="S11" s="93"/>
-      <c r="T11" s="93"/>
-      <c r="U11" s="93"/>
-      <c r="V11" s="93"/>
-      <c r="W11" s="93"/>
+      <c r="S11" s="48"/>
+      <c r="T11" s="48"/>
+      <c r="U11" s="48"/>
+      <c r="V11" s="48"/>
+      <c r="W11" s="48"/>
     </row>
     <row r="12" ht="14.25" spans="1:23">
-      <c r="A12" s="14" t="s">
+      <c r="A12" s="31" t="s">
         <v>20</v>
       </c>
-      <c r="B12" s="15"/>
-      <c r="C12" s="16"/>
-      <c r="D12" s="17"/>
-      <c r="E12" s="18" t="s">
+      <c r="B12" s="32"/>
+      <c r="C12" s="33"/>
+      <c r="D12" s="34"/>
+      <c r="E12" s="35" t="s">
         <v>61</v>
       </c>
-      <c r="F12" s="18" t="s">
+      <c r="F12" s="35" t="s">
         <v>62</v>
       </c>
-      <c r="G12" s="20" t="s">
+      <c r="G12" s="49" t="s">
         <v>63</v>
       </c>
-      <c r="H12" s="18" t="s">
+      <c r="H12" s="35" t="s">
         <v>46</v>
       </c>
-      <c r="I12" s="20" t="s">
+      <c r="I12" s="49" t="s">
         <v>12</v>
       </c>
-      <c r="J12" s="63"/>
-      <c r="L12" s="68" t="s">
+      <c r="J12" s="36"/>
+      <c r="L12" s="50" t="s">
         <v>64</v>
       </c>
-      <c r="M12" s="68"/>
-      <c r="N12" s="68"/>
-      <c r="O12" s="68"/>
-      <c r="P12" s="68"/>
-      <c r="R12" s="68" t="s">
+      <c r="M12" s="50"/>
+      <c r="N12" s="50"/>
+      <c r="O12" s="50"/>
+      <c r="P12" s="50"/>
+      <c r="R12" s="50" t="s">
         <v>64</v>
       </c>
-      <c r="S12" s="68"/>
-      <c r="T12" s="68"/>
-      <c r="U12" s="68"/>
-      <c r="V12" s="68"/>
-      <c r="W12" s="68"/>
+      <c r="S12" s="50"/>
+      <c r="T12" s="50"/>
+      <c r="U12" s="50"/>
+      <c r="V12" s="50"/>
+      <c r="W12" s="50"/>
     </row>
     <row r="13" ht="14.25" spans="1:23">
-      <c r="A13" s="21" t="s">
+      <c r="A13" s="51" t="s">
         <v>65</v>
       </c>
-      <c r="B13" s="22"/>
-      <c r="C13" s="23"/>
-      <c r="D13" s="24"/>
-      <c r="E13" s="25" t="s">
+      <c r="B13" s="52"/>
+      <c r="C13" s="53"/>
+      <c r="D13" s="54"/>
+      <c r="E13" s="55" t="s">
         <v>66</v>
       </c>
-      <c r="F13" s="25">
+      <c r="F13" s="55">
         <v>5</v>
       </c>
-      <c r="G13" s="26" t="s">
+      <c r="G13" s="56" t="s">
         <v>67</v>
       </c>
-      <c r="H13" s="27" t="s">
+      <c r="H13" s="57" t="s">
         <v>68</v>
       </c>
-      <c r="I13" s="27"/>
-      <c r="J13" s="69"/>
-      <c r="L13" s="70"/>
-      <c r="M13" s="70" t="s">
+      <c r="I13" s="57"/>
+      <c r="J13" s="58"/>
+      <c r="L13" s="59"/>
+      <c r="M13" s="59" t="s">
         <v>69</v>
       </c>
-      <c r="N13" s="70"/>
-      <c r="O13" s="70"/>
-      <c r="P13" s="70"/>
-      <c r="R13" s="70"/>
-      <c r="S13" s="70" t="s">
+      <c r="N13" s="59"/>
+      <c r="O13" s="59"/>
+      <c r="P13" s="59"/>
+      <c r="R13" s="59"/>
+      <c r="S13" s="59" t="s">
         <v>70</v>
       </c>
-      <c r="T13" s="70"/>
-      <c r="U13" s="50" t="s">
+      <c r="T13" s="59"/>
+      <c r="U13" s="60" t="s">
         <v>71</v>
       </c>
-      <c r="V13" s="50"/>
-      <c r="W13" s="50"/>
-    </row>
-    <row r="14" ht="14.25" spans="2:23">
+      <c r="V13" s="60"/>
+      <c r="W13" s="60"/>
+    </row>
+    <row r="14" ht="14.25" spans="1:23">
       <c r="B14" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="L14" s="70"/>
-      <c r="M14" s="70" t="s">
+      <c r="L14" s="59"/>
+      <c r="M14" s="59" t="s">
         <v>73</v>
       </c>
-      <c r="N14" s="70"/>
-      <c r="O14" s="70"/>
-      <c r="P14" s="70"/>
-      <c r="R14" s="70"/>
-      <c r="S14" s="70" t="s">
+      <c r="N14" s="59"/>
+      <c r="O14" s="59"/>
+      <c r="P14" s="59"/>
+      <c r="R14" s="59"/>
+      <c r="S14" s="59" t="s">
         <v>74</v>
       </c>
-      <c r="T14" s="70"/>
-      <c r="U14" s="50" t="s">
+      <c r="T14" s="59"/>
+      <c r="U14" s="60" t="s">
         <v>75</v>
       </c>
-      <c r="V14" s="50"/>
-      <c r="W14" s="50"/>
-    </row>
-    <row r="15" spans="12:23">
-      <c r="L15" s="70"/>
-      <c r="M15" s="70" t="s">
+      <c r="V14" s="60"/>
+      <c r="W14" s="60"/>
+    </row>
+    <row r="15" spans="1:23">
+      <c r="L15" s="59"/>
+      <c r="M15" s="59" t="s">
         <v>76</v>
       </c>
-      <c r="N15" s="70"/>
-      <c r="O15" s="70"/>
-      <c r="P15" s="70"/>
-      <c r="R15" s="70"/>
-      <c r="S15" s="70" t="s">
+      <c r="N15" s="59"/>
+      <c r="O15" s="59"/>
+      <c r="P15" s="59"/>
+      <c r="R15" s="59"/>
+      <c r="S15" s="59" t="s">
         <v>77</v>
       </c>
-      <c r="T15" s="70"/>
-      <c r="U15" s="50" t="s">
+      <c r="T15" s="59"/>
+      <c r="U15" s="60" t="s">
         <v>78</v>
       </c>
-      <c r="V15" s="50"/>
-      <c r="W15" s="50"/>
-    </row>
-    <row r="16" ht="14.25" spans="12:23">
-      <c r="L16" s="70"/>
-      <c r="M16" s="70" t="s">
+      <c r="V15" s="60"/>
+      <c r="W15" s="60"/>
+    </row>
+    <row r="16" ht="14.25" spans="1:23">
+      <c r="L16" s="59"/>
+      <c r="M16" s="59" t="s">
         <v>79</v>
       </c>
-      <c r="N16" s="70"/>
-      <c r="O16" s="70"/>
-      <c r="P16" s="70"/>
-      <c r="R16" s="70"/>
-      <c r="S16" s="70" t="s">
+      <c r="N16" s="59"/>
+      <c r="O16" s="59"/>
+      <c r="P16" s="59"/>
+      <c r="R16" s="59"/>
+      <c r="S16" s="59" t="s">
         <v>80</v>
       </c>
-      <c r="T16" s="70"/>
-      <c r="U16" s="50" t="s">
+      <c r="T16" s="59"/>
+      <c r="U16" s="60" t="s">
         <v>81</v>
       </c>
-      <c r="V16" s="50"/>
-      <c r="W16" s="50"/>
-    </row>
-    <row r="17" s="1" customFormat="1" ht="15" spans="1:10">
-      <c r="A17" s="28" t="s">
+      <c r="V16" s="60"/>
+      <c r="W16" s="60"/>
+    </row>
+    <row r="17" s="1" customFormat="1" ht="15" spans="1:19">
+      <c r="A17" s="61" t="s">
         <v>82</v>
       </c>
-      <c r="B17" s="28"/>
-      <c r="C17" s="28"/>
-      <c r="D17" s="28"/>
-      <c r="E17" s="28"/>
-      <c r="F17" s="28"/>
-      <c r="G17" s="28"/>
-      <c r="H17" s="28"/>
-      <c r="I17" s="28"/>
-      <c r="J17" s="28"/>
-    </row>
-    <row r="18" ht="15" spans="1:10">
-      <c r="A18" s="29"/>
-      <c r="B18" s="29" t="s">
+      <c r="B17" s="61"/>
+      <c r="C17" s="61"/>
+      <c r="D17" s="61"/>
+      <c r="E17" s="61"/>
+      <c r="F17" s="61"/>
+      <c r="G17" s="61"/>
+      <c r="H17" s="61"/>
+      <c r="I17" s="61"/>
+      <c r="J17" s="61"/>
+    </row>
+    <row r="18" ht="15" spans="1:19">
+      <c r="A18" s="62"/>
+      <c r="B18" s="62" t="s">
         <v>4</v>
       </c>
-      <c r="C18" s="29" t="s">
+      <c r="C18" s="62" t="s">
         <v>5</v>
       </c>
-      <c r="D18" s="29" t="s">
+      <c r="D18" s="62" t="s">
         <v>6</v>
       </c>
-      <c r="E18" s="29" t="s">
+      <c r="E18" s="62" t="s">
         <v>7</v>
       </c>
-      <c r="F18" s="29" t="s">
+      <c r="F18" s="62" t="s">
         <v>8</v>
       </c>
-      <c r="G18" s="29" t="s">
+      <c r="G18" s="62" t="s">
         <v>83</v>
       </c>
-      <c r="H18" s="29"/>
-      <c r="I18" s="29"/>
-      <c r="J18" s="29" t="s">
+      <c r="H18" s="62"/>
+      <c r="I18" s="62"/>
+      <c r="J18" s="62" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="19" ht="15" spans="1:10">
-      <c r="A19" s="29"/>
-      <c r="B19" s="30" t="s">
+    <row r="19" ht="15" spans="1:19">
+      <c r="A19" s="62"/>
+      <c r="B19" s="63" t="s">
         <v>13</v>
       </c>
-      <c r="C19" s="30" t="s">
+      <c r="C19" s="63" t="s">
         <v>14</v>
       </c>
-      <c r="D19" s="30" t="s">
+      <c r="D19" s="63" t="s">
         <v>15</v>
       </c>
-      <c r="E19" s="30" t="s">
+      <c r="E19" s="63" t="s">
         <v>15</v>
       </c>
-      <c r="F19" s="30" t="s">
+      <c r="F19" s="63" t="s">
         <v>13</v>
       </c>
-      <c r="G19" s="30" t="s">
+      <c r="G19" s="63" t="s">
         <v>15</v>
       </c>
-      <c r="H19" s="30"/>
-      <c r="I19" s="30"/>
-      <c r="J19" s="30" t="s">
+      <c r="H19" s="63"/>
+      <c r="I19" s="63"/>
+      <c r="J19" s="63" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="20" s="2" customFormat="1" ht="15" spans="1:10">
-      <c r="A20" s="31" t="s">
+    <row r="20" s="2" customFormat="1" ht="15" spans="1:19">
+      <c r="A20" s="64" t="s">
         <v>84</v>
       </c>
-      <c r="B20" s="32" t="s">
+      <c r="B20" s="65" t="s">
         <v>85</v>
       </c>
-      <c r="C20" s="33" t="s">
+      <c r="C20" s="66" t="s">
         <v>33</v>
       </c>
-      <c r="D20" s="34" t="s">
+      <c r="D20" s="67" t="s">
         <v>24</v>
       </c>
-      <c r="E20" s="35" t="s">
+      <c r="E20" s="68" t="s">
         <v>25</v>
       </c>
-      <c r="F20" s="35">
+      <c r="F20" s="68">
         <v>4</v>
       </c>
-      <c r="G20" s="35" t="s">
+      <c r="G20" s="68" t="s">
         <v>86</v>
       </c>
-      <c r="H20" s="35"/>
-      <c r="I20" s="35"/>
-      <c r="J20" s="71" t="s">
+      <c r="H20" s="68"/>
+      <c r="I20" s="68"/>
+      <c r="J20" s="69" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="21" ht="14.25" spans="1:10">
-      <c r="A21" s="14" t="s">
+    <row r="21" ht="14.25" spans="1:19">
+      <c r="A21" s="31" t="s">
         <v>87</v>
       </c>
-      <c r="B21" s="36"/>
-      <c r="C21" s="16"/>
-      <c r="D21" s="17"/>
-      <c r="E21" s="18" t="s">
+      <c r="B21" s="70"/>
+      <c r="C21" s="33"/>
+      <c r="D21" s="34"/>
+      <c r="E21" s="35" t="s">
         <v>34</v>
       </c>
-      <c r="F21" s="18">
+      <c r="F21" s="35">
         <v>1</v>
       </c>
-      <c r="G21" s="18" t="s">
+      <c r="G21" s="35" t="s">
         <v>88</v>
       </c>
-      <c r="H21" s="18"/>
-      <c r="I21" s="18"/>
-      <c r="J21" s="71"/>
-    </row>
-    <row r="22" ht="14.25" spans="1:10">
-      <c r="A22" s="14" t="s">
+      <c r="H21" s="35"/>
+      <c r="I21" s="35"/>
+      <c r="J21" s="69"/>
+    </row>
+    <row r="22" ht="14.25" spans="1:19">
+      <c r="A22" s="31" t="s">
         <v>89</v>
       </c>
-      <c r="B22" s="36"/>
-      <c r="C22" s="16"/>
-      <c r="D22" s="17"/>
-      <c r="E22" s="18" t="s">
+      <c r="B22" s="70"/>
+      <c r="C22" s="33"/>
+      <c r="D22" s="34"/>
+      <c r="E22" s="35" t="s">
         <v>41</v>
       </c>
-      <c r="F22" s="18">
+      <c r="F22" s="35">
         <v>1</v>
       </c>
-      <c r="G22" s="18" t="s">
+      <c r="G22" s="35" t="s">
         <v>88</v>
       </c>
-      <c r="H22" s="18"/>
-      <c r="I22" s="18"/>
-      <c r="J22" s="71"/>
+      <c r="H22" s="35"/>
+      <c r="I22" s="35"/>
+      <c r="J22" s="69"/>
     </row>
     <row r="23" ht="14.25" spans="1:19">
-      <c r="A23" s="14" t="s">
+      <c r="A23" s="31" t="s">
         <v>90</v>
       </c>
-      <c r="B23" s="36"/>
-      <c r="C23" s="16"/>
-      <c r="D23" s="17"/>
-      <c r="E23" s="18" t="s">
+      <c r="B23" s="70"/>
+      <c r="C23" s="33"/>
+      <c r="D23" s="34"/>
+      <c r="E23" s="35" t="s">
         <v>49</v>
       </c>
-      <c r="F23" s="18">
+      <c r="F23" s="35">
         <v>1</v>
       </c>
-      <c r="G23" s="18" t="s">
+      <c r="G23" s="35" t="s">
         <v>88</v>
       </c>
-      <c r="H23" s="18"/>
-      <c r="I23" s="18"/>
-      <c r="J23" s="71"/>
-      <c r="R23" s="51"/>
-      <c r="S23" s="51"/>
+      <c r="H23" s="35"/>
+      <c r="I23" s="35"/>
+      <c r="J23" s="69"/>
+      <c r="R23" s="4"/>
+      <c r="S23" s="4"/>
     </row>
     <row r="24" ht="14.25" spans="1:19">
-      <c r="A24" s="14" t="s">
+      <c r="A24" s="31" t="s">
         <v>91</v>
       </c>
-      <c r="B24" s="36"/>
-      <c r="C24" s="16"/>
-      <c r="D24" s="17"/>
-      <c r="E24" s="18" t="s">
+      <c r="B24" s="70"/>
+      <c r="C24" s="33"/>
+      <c r="D24" s="34"/>
+      <c r="E24" s="35" t="s">
         <v>52</v>
       </c>
-      <c r="F24" s="18">
+      <c r="F24" s="35">
         <v>1</v>
       </c>
-      <c r="G24" s="18" t="s">
+      <c r="G24" s="35" t="s">
         <v>92</v>
       </c>
-      <c r="H24" s="18"/>
-      <c r="I24" s="18"/>
-      <c r="J24" s="71"/>
-      <c r="R24" s="51"/>
-      <c r="S24" s="51"/>
+      <c r="H24" s="35"/>
+      <c r="I24" s="35"/>
+      <c r="J24" s="69"/>
+      <c r="R24" s="4"/>
+      <c r="S24" s="4"/>
     </row>
     <row r="25" ht="14.25" spans="1:19">
-      <c r="A25" s="14" t="s">
+      <c r="A25" s="31" t="s">
         <v>93</v>
       </c>
-      <c r="B25" s="36"/>
-      <c r="C25" s="16"/>
-      <c r="D25" s="17"/>
-      <c r="E25" s="18" t="s">
+      <c r="B25" s="70"/>
+      <c r="C25" s="33"/>
+      <c r="D25" s="34"/>
+      <c r="E25" s="35" t="s">
         <v>56</v>
       </c>
-      <c r="F25" s="18">
+      <c r="F25" s="35">
         <v>1</v>
       </c>
-      <c r="G25" s="18" t="s">
+      <c r="G25" s="35" t="s">
         <v>88</v>
       </c>
-      <c r="H25" s="18"/>
-      <c r="I25" s="18"/>
-      <c r="J25" s="71"/>
-      <c r="R25" s="51"/>
-      <c r="S25" s="51"/>
+      <c r="H25" s="35"/>
+      <c r="I25" s="35"/>
+      <c r="J25" s="69"/>
+      <c r="R25" s="4"/>
+      <c r="S25" s="4"/>
     </row>
     <row r="26" ht="14.25" spans="1:19">
-      <c r="A26" s="21" t="s">
+      <c r="A26" s="51" t="s">
         <v>94</v>
       </c>
-      <c r="B26" s="37"/>
-      <c r="C26" s="23"/>
-      <c r="D26" s="24"/>
-      <c r="E26" s="25" t="s">
+      <c r="B26" s="71"/>
+      <c r="C26" s="53"/>
+      <c r="D26" s="54"/>
+      <c r="E26" s="55" t="s">
         <v>61</v>
       </c>
-      <c r="F26" s="25">
+      <c r="F26" s="55">
         <v>1</v>
       </c>
-      <c r="G26" s="25" t="s">
+      <c r="G26" s="55" t="s">
         <v>88</v>
       </c>
-      <c r="H26" s="25"/>
-      <c r="I26" s="25"/>
+      <c r="H26" s="55"/>
+      <c r="I26" s="55"/>
       <c r="J26" s="72"/>
-      <c r="R26" s="94"/>
-      <c r="S26" s="94"/>
+      <c r="R26" s="73"/>
+      <c r="S26" s="73"/>
     </row>
     <row r="27" ht="15"/>
-    <row r="28" s="1" customFormat="1" ht="15" spans="1:13">
-      <c r="A28" s="38" t="s">
+    <row r="28" s="1" customFormat="1" ht="15" spans="1:19">
+      <c r="A28" s="74" t="s">
         <v>95</v>
       </c>
-      <c r="B28" s="39"/>
-      <c r="C28" s="39"/>
-      <c r="D28" s="39"/>
-      <c r="E28" s="39"/>
-      <c r="F28" s="39"/>
-      <c r="G28" s="39"/>
-      <c r="H28" s="39"/>
-      <c r="I28" s="39"/>
-      <c r="J28" s="39"/>
-      <c r="K28" s="73"/>
-      <c r="M28" s="74"/>
-    </row>
-    <row r="29" ht="15" spans="1:11">
-      <c r="A29" s="6"/>
-      <c r="B29" s="6" t="s">
+      <c r="B28" s="75"/>
+      <c r="C28" s="75"/>
+      <c r="D28" s="75"/>
+      <c r="E28" s="75"/>
+      <c r="F28" s="75"/>
+      <c r="G28" s="75"/>
+      <c r="H28" s="75"/>
+      <c r="I28" s="75"/>
+      <c r="J28" s="75"/>
+      <c r="K28" s="76"/>
+      <c r="M28" s="77"/>
+    </row>
+    <row r="29" ht="15" spans="1:19">
+      <c r="A29" s="11"/>
+      <c r="B29" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="C29" s="6" t="s">
+      <c r="C29" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="D29" s="6" t="s">
+      <c r="D29" s="11" t="s">
         <v>96</v>
       </c>
-      <c r="E29" s="6" t="s">
+      <c r="E29" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="F29" s="6" t="s">
+      <c r="F29" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="G29" s="6" t="s">
+      <c r="G29" s="11" t="s">
         <v>83</v>
       </c>
-      <c r="H29" s="6"/>
-      <c r="I29" s="75"/>
-      <c r="J29" s="6" t="s">
+      <c r="H29" s="11"/>
+      <c r="I29" s="78"/>
+      <c r="J29" s="11" t="s">
         <v>97</v>
       </c>
-      <c r="K29" s="76" t="s">
+      <c r="K29" s="79" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="30" ht="15" spans="1:11">
-      <c r="A30" s="29"/>
-      <c r="B30" s="30" t="s">
+    <row r="30" ht="15" spans="1:19">
+      <c r="A30" s="62"/>
+      <c r="B30" s="63" t="s">
         <v>13</v>
       </c>
-      <c r="C30" s="30" t="s">
+      <c r="C30" s="63" t="s">
         <v>14</v>
       </c>
-      <c r="D30" s="30" t="s">
+      <c r="D30" s="63" t="s">
         <v>15</v>
       </c>
-      <c r="E30" s="30" t="s">
+      <c r="E30" s="63" t="s">
         <v>15</v>
       </c>
-      <c r="F30" s="30" t="s">
+      <c r="F30" s="63" t="s">
         <v>13</v>
       </c>
-      <c r="G30" s="30" t="s">
+      <c r="G30" s="63" t="s">
         <v>98</v>
       </c>
-      <c r="H30" s="30"/>
-      <c r="I30" s="77"/>
-      <c r="J30" s="30" t="s">
+      <c r="H30" s="63"/>
+      <c r="I30" s="80"/>
+      <c r="J30" s="63" t="s">
         <v>99</v>
       </c>
-      <c r="K30" s="78" t="s">
+      <c r="K30" s="81" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="31" ht="30" customHeight="1" spans="1:11">
-      <c r="A31" s="31" t="s">
+    <row r="31" ht="30" customHeight="1" spans="1:19">
+      <c r="A31" s="64" t="s">
         <v>100</v>
       </c>
-      <c r="B31" s="40" t="s">
+      <c r="B31" s="82" t="s">
         <v>85</v>
       </c>
-      <c r="C31" s="33" t="s">
+      <c r="C31" s="66" t="s">
         <v>33</v>
       </c>
-      <c r="D31" s="34" t="s">
+      <c r="D31" s="67" t="s">
         <v>101</v>
       </c>
-      <c r="E31" s="35" t="s">
+      <c r="E31" s="68" t="s">
         <v>102</v>
       </c>
-      <c r="F31" s="35" t="s">
+      <c r="F31" s="68" t="s">
         <v>103</v>
       </c>
-      <c r="G31" s="41" t="s">
+      <c r="G31" s="83" t="s">
         <v>104</v>
       </c>
-      <c r="H31" s="42"/>
-      <c r="I31" s="79"/>
-      <c r="J31" s="80" t="s">
+      <c r="H31" s="84"/>
+      <c r="I31" s="85"/>
+      <c r="J31" s="86" t="s">
         <v>97</v>
       </c>
-      <c r="K31" s="71" t="s">
+      <c r="K31" s="69" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="32" ht="30" customHeight="1" spans="1:11">
-      <c r="A32" s="21" t="s">
+    <row r="32" ht="30" customHeight="1" spans="1:19">
+      <c r="A32" s="51" t="s">
         <v>105</v>
       </c>
-      <c r="B32" s="43"/>
-      <c r="C32" s="23"/>
-      <c r="D32" s="25"/>
-      <c r="E32" s="25" t="s">
+      <c r="B32" s="87"/>
+      <c r="C32" s="53"/>
+      <c r="D32" s="55"/>
+      <c r="E32" s="55" t="s">
         <v>66</v>
       </c>
-      <c r="F32" s="25" t="s">
+      <c r="F32" s="55" t="s">
         <v>103</v>
       </c>
-      <c r="G32" s="44"/>
-      <c r="H32" s="45"/>
-      <c r="I32" s="45"/>
-      <c r="J32" s="80"/>
+      <c r="G32" s="88"/>
+      <c r="H32" s="89"/>
+      <c r="I32" s="89"/>
+      <c r="J32" s="86"/>
       <c r="K32" s="72"/>
     </row>
     <row r="33" ht="14.25"/>
-    <row r="34" spans="1:17">
-      <c r="A34" s="46" t="s">
+    <row r="34" spans="1:18">
+      <c r="A34" s="90" t="s">
         <v>106</v>
       </c>
-      <c r="B34" s="46"/>
-      <c r="C34" s="46"/>
-      <c r="D34" s="46"/>
-      <c r="E34" s="46"/>
-      <c r="F34" s="46"/>
-      <c r="G34" s="46"/>
-      <c r="H34" s="46"/>
-      <c r="I34" s="46"/>
-      <c r="J34" s="46"/>
-      <c r="K34" s="46"/>
-      <c r="L34" s="81"/>
-      <c r="M34" s="81"/>
-      <c r="N34" s="81"/>
-      <c r="O34" s="81"/>
-      <c r="P34" s="81"/>
-      <c r="Q34" s="81"/>
-    </row>
-    <row r="35" spans="1:17">
-      <c r="A35" s="46" t="s">
+      <c r="B34" s="90"/>
+      <c r="C34" s="90"/>
+      <c r="D34" s="90"/>
+      <c r="E34" s="90"/>
+      <c r="F34" s="90"/>
+      <c r="G34" s="90"/>
+      <c r="H34" s="90"/>
+      <c r="I34" s="90"/>
+      <c r="J34" s="90"/>
+      <c r="K34" s="90"/>
+      <c r="L34" s="91"/>
+      <c r="M34" s="91"/>
+      <c r="N34" s="91"/>
+      <c r="O34" s="91"/>
+      <c r="P34" s="91"/>
+      <c r="Q34" s="91"/>
+    </row>
+    <row r="35" spans="1:18">
+      <c r="A35" s="90" t="s">
         <v>107</v>
       </c>
-      <c r="B35" s="46"/>
-      <c r="C35" s="46"/>
-      <c r="D35" s="46"/>
-      <c r="E35" s="46"/>
-      <c r="F35" s="46"/>
-      <c r="G35" s="46"/>
-      <c r="H35" s="46"/>
-      <c r="I35" s="46"/>
-      <c r="J35" s="46"/>
-      <c r="K35" s="46"/>
-      <c r="L35" s="81"/>
-      <c r="M35" s="81"/>
-      <c r="N35" s="81"/>
-      <c r="O35" s="81"/>
-      <c r="P35" s="81"/>
-      <c r="Q35" s="81"/>
-    </row>
-    <row r="36" spans="1:17">
-      <c r="A36" s="47"/>
-      <c r="B36" s="47"/>
-      <c r="C36" s="47"/>
-      <c r="D36" s="47"/>
-      <c r="E36" s="47"/>
-      <c r="F36" s="47"/>
-      <c r="G36" s="47"/>
-      <c r="H36" s="47"/>
-      <c r="I36" s="47"/>
-      <c r="J36" s="47"/>
-      <c r="K36" s="47"/>
-      <c r="L36" s="47"/>
-      <c r="M36" s="47"/>
-      <c r="N36" s="47"/>
-      <c r="O36" s="47"/>
-      <c r="P36" s="47"/>
-      <c r="Q36" s="47"/>
+      <c r="B35" s="90"/>
+      <c r="C35" s="90"/>
+      <c r="D35" s="90"/>
+      <c r="E35" s="90"/>
+      <c r="F35" s="90"/>
+      <c r="G35" s="90"/>
+      <c r="H35" s="90"/>
+      <c r="I35" s="90"/>
+      <c r="J35" s="90"/>
+      <c r="K35" s="90"/>
+      <c r="L35" s="91"/>
+      <c r="M35" s="91"/>
+      <c r="N35" s="91"/>
+      <c r="O35" s="91"/>
+      <c r="P35" s="91"/>
+      <c r="Q35" s="91"/>
+    </row>
+    <row r="36" spans="1:18">
+      <c r="A36" s="92"/>
+      <c r="B36" s="92"/>
+      <c r="C36" s="92"/>
+      <c r="D36" s="92"/>
+      <c r="E36" s="92"/>
+      <c r="F36" s="92"/>
+      <c r="G36" s="92"/>
+      <c r="H36" s="92"/>
+      <c r="I36" s="92"/>
+      <c r="J36" s="92"/>
+      <c r="K36" s="92"/>
+      <c r="L36" s="92"/>
+      <c r="M36" s="92"/>
+      <c r="N36" s="92"/>
+      <c r="O36" s="92"/>
+      <c r="P36" s="92"/>
+      <c r="Q36" s="92"/>
     </row>
     <row r="37" spans="1:18">
-      <c r="A37" s="48" t="s">
+      <c r="A37" s="93" t="s">
         <v>108</v>
       </c>
-      <c r="B37" s="49"/>
-      <c r="C37" s="49"/>
-      <c r="D37" s="49"/>
-      <c r="E37" s="49"/>
-      <c r="F37" s="49"/>
-      <c r="G37" s="49"/>
-      <c r="H37" s="49"/>
-      <c r="I37" s="49"/>
-      <c r="J37" s="49"/>
-      <c r="K37" s="49"/>
-      <c r="L37" s="49"/>
-      <c r="M37" s="49"/>
-      <c r="N37" s="49"/>
-      <c r="O37" s="49"/>
-      <c r="P37" s="49"/>
-      <c r="Q37" s="49"/>
+      <c r="B37" s="94"/>
+      <c r="C37" s="94"/>
+      <c r="D37" s="94"/>
+      <c r="E37" s="94"/>
+      <c r="F37" s="94"/>
+      <c r="G37" s="94"/>
+      <c r="H37" s="94"/>
+      <c r="I37" s="94"/>
+      <c r="J37" s="94"/>
+      <c r="K37" s="94"/>
+      <c r="L37" s="94"/>
+      <c r="M37" s="94"/>
+      <c r="N37" s="94"/>
+      <c r="O37" s="94"/>
+      <c r="P37" s="94"/>
+      <c r="Q37" s="94"/>
       <c r="R37" s="95"/>
     </row>
     <row r="38" spans="1:18">
-      <c r="A38" s="50" t="s">
+      <c r="A38" s="60" t="s">
         <v>109</v>
       </c>
-      <c r="B38" s="50"/>
-      <c r="C38" s="50"/>
-      <c r="D38" s="50"/>
-      <c r="E38" s="50"/>
-      <c r="F38" s="50"/>
-      <c r="G38" s="50"/>
-      <c r="H38" s="50"/>
-      <c r="I38" s="50"/>
-      <c r="J38" s="50"/>
-      <c r="K38" s="50"/>
-      <c r="L38" s="50"/>
-      <c r="M38" s="50"/>
-      <c r="N38" s="50"/>
-      <c r="O38" s="50"/>
-      <c r="P38" s="50"/>
-      <c r="Q38" s="50"/>
-      <c r="R38" s="50"/>
+      <c r="B38" s="60"/>
+      <c r="C38" s="60"/>
+      <c r="D38" s="60"/>
+      <c r="E38" s="60"/>
+      <c r="F38" s="60"/>
+      <c r="G38" s="60"/>
+      <c r="H38" s="60"/>
+      <c r="I38" s="60"/>
+      <c r="J38" s="60"/>
+      <c r="K38" s="60"/>
+      <c r="L38" s="60"/>
+      <c r="M38" s="60"/>
+      <c r="N38" s="60"/>
+      <c r="O38" s="60"/>
+      <c r="P38" s="60"/>
+      <c r="Q38" s="60"/>
+      <c r="R38" s="60"/>
     </row>
     <row r="39" spans="1:18">
-      <c r="A39" s="50" t="s">
+      <c r="A39" s="60" t="s">
         <v>110</v>
       </c>
-      <c r="B39" s="50"/>
-      <c r="C39" s="50"/>
-      <c r="D39" s="50"/>
-      <c r="E39" s="50"/>
-      <c r="F39" s="50"/>
-      <c r="G39" s="50"/>
-      <c r="H39" s="50"/>
-      <c r="I39" s="50"/>
-      <c r="J39" s="50"/>
-      <c r="K39" s="50"/>
-      <c r="L39" s="50"/>
-      <c r="M39" s="50"/>
-      <c r="N39" s="50"/>
-      <c r="O39" s="50"/>
-      <c r="P39" s="50"/>
-      <c r="Q39" s="50"/>
-      <c r="R39" s="50"/>
+      <c r="B39" s="60"/>
+      <c r="C39" s="60"/>
+      <c r="D39" s="60"/>
+      <c r="E39" s="60"/>
+      <c r="F39" s="60"/>
+      <c r="G39" s="60"/>
+      <c r="H39" s="60"/>
+      <c r="I39" s="60"/>
+      <c r="J39" s="60"/>
+      <c r="K39" s="60"/>
+      <c r="L39" s="60"/>
+      <c r="M39" s="60"/>
+      <c r="N39" s="60"/>
+      <c r="O39" s="60"/>
+      <c r="P39" s="60"/>
+      <c r="Q39" s="60"/>
+      <c r="R39" s="60"/>
     </row>
   </sheetData>
   <mergeCells count="71">

</xml_diff>